<commit_message>
Stage 8 review fixes: F-013
</commit_message>
<xml_diff>
--- a/output/archive/DurnesswickData/Development/WX19/Vehicle_Optimisation/Bench_Sheets/WX19_physical-stability_020926_hold.xlsx
+++ b/output/archive/DurnesswickData/Development/WX19/Vehicle_Optimisation/Bench_Sheets/WX19_physical-stability_020926_hold.xlsx
@@ -828,7 +828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -840,7 +840,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Physical stability, 10 mg/mL suspensions, observation log</t>
+          <t>Physical stability follow-up: observation tracker</t>
         </is>
       </c>
     </row>
@@ -852,12 +852,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Read date</t>
+          <t>Next read date</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Observation</t>
+          <t>Follow-up observation</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -872,21 +872,9 @@
           <t>0.5% methylcellulose</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>02/09/2026</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Settles, redispersible on shaking</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>M. Serrano</t>
-        </is>
-      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -894,21 +882,9 @@
           <t>0.5% HPMC / 0.1% Tween 80</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>02/09/2026</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Caking at the bottom of the vial</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>M. Serrano</t>
-        </is>
-      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -916,62 +892,32 @@
           <t>20% HP-β-CD in water</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>02/09/2026</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Caking, hard to redisperse</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>M. Serrano</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>0.5% methylcellulose</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-    </row>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>0.5% HPMC / 0.1% Tween 80</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
+          <t>Initial observations</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>See the vehicle screen for the 24 h observations.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>20% HP-β-CD in water</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Next read</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Due after the hold is lifted. Dates not set.</t>
+          <t>Ongoing observation</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Samples remain under observation during the optimisation hold. Subsequent reads belong in the source observation log.</t>
         </is>
       </c>
     </row>
@@ -1032,7 +978,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Option A</t>
+          <t>Pending client decision</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
@@ -1040,21 +986,13 @@
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Option B</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr"/>
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Option C</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr"/>
@@ -1119,7 +1057,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Optimisation paused at Wexanthel's request until the flavour panel decision. No further work is booked on this work package.</t>
+          <t>Optimisation paused at Wexanthel's request pending its flavour-panel decision. Physical stability observations continue separately.</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1069,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Samples retained under observation. Next read to be booked when the hold is lifted.</t>
+          <t>Samples remain under observation; subsequent readings belong in the source observation log. No final vehicle recommendation is issued.</t>
         </is>
       </c>
     </row>

</xml_diff>